<commit_message>
import setup for FE & BE, merge single subject score
</commit_message>
<xml_diff>
--- a/backend/test/excel/Book1.xlsx
+++ b/backend/test/excel/Book1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tri/Documents/Work/GoEasy/backend/test/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973D3DE5-8731-6349-B136-D34B3545CF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8320B1D8-862C-8C48-9FD8-815467977A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="0" windowWidth="28040" windowHeight="17440" xr2:uid="{D1F6A292-1550-A549-9D17-35C903551DCF}"/>
+    <workbookView xWindow="5280" yWindow="320" windowWidth="28040" windowHeight="17440" xr2:uid="{D1F6A292-1550-A549-9D17-35C903551DCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Trần Văn A</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>Anh</t>
-  </si>
-  <si>
-    <t>TB</t>
   </si>
 </sst>
 </file>
@@ -439,63 +436,25 @@
       <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>5</v>
-      </c>
-      <c r="E2" s="2">
-        <f t="shared" ref="E2:E3" si="0">AVERAGE(B2:D2)</f>
-        <v>3.3333333333333335</v>
-      </c>
+      <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
-        <v>6.5</v>
-      </c>
-      <c r="C3">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2">
-        <f t="shared" si="0"/>
-        <v>8.1666666666666661</v>
-      </c>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="D4">
-        <v>9</v>
-      </c>
-      <c r="E4" s="2">
-        <f>AVERAGE(B4:D4)</f>
-        <v>8.8333333333333339</v>
-      </c>
+      <c r="C4" s="1"/>
+      <c r="E4" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>